<commit_message>
Add basic test for regional analysis
</commit_message>
<xml_diff>
--- a/individual image/first-image/5000/5000 - Regional Analysis.xlsx
+++ b/individual image/first-image/5000/5000 - Regional Analysis.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Regional analysis_Square Grid" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Regional analysis_ETDRS Grid" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Regional analysis_Square grid" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Regional analysis_ETDRS grid" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Regional analysis_Extended ETDR" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Regional analysis_Foveal Ring" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Regional analysis_ONH" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Regional analysis_Foveal rings" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Regional analysis_Optic nerve h" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -506,25 +506,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C2" t="n">
         <v>33.92</v>
       </c>
       <c r="D2" t="n">
-        <v>20.01</v>
+        <v>20</v>
       </c>
       <c r="E2" t="n">
-        <v>6.02</v>
+        <v>6.01</v>
       </c>
       <c r="F2" t="n">
-        <v>20.0504</v>
+        <v>20.0369</v>
       </c>
       <c r="G2" t="n">
         <v>70</v>
       </c>
       <c r="H2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I2" t="n">
         <v>19</v>
@@ -533,13 +533,13 @@
         <v>18</v>
       </c>
       <c r="K2" t="n">
-        <v>5.6</v>
+        <v>5.65</v>
       </c>
       <c r="L2" t="n">
-        <v>1.4282</v>
+        <v>1.4298</v>
       </c>
       <c r="M2" t="n">
-        <v>1.2115</v>
+        <v>1.2134</v>
       </c>
     </row>
     <row r="3">
@@ -549,25 +549,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C3" t="n">
         <v>36.44</v>
       </c>
       <c r="D3" t="n">
-        <v>22.72</v>
+        <v>22.84</v>
       </c>
       <c r="E3" t="n">
-        <v>6.83</v>
+        <v>6.87</v>
       </c>
       <c r="F3" t="n">
-        <v>22.7621</v>
+        <v>22.8844</v>
       </c>
       <c r="G3" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H3" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I3" t="n">
         <v>17</v>
@@ -576,13 +576,13 @@
         <v>17</v>
       </c>
       <c r="K3" t="n">
-        <v>7</v>
+        <v>6.87</v>
       </c>
       <c r="L3" t="n">
-        <v>1.4527</v>
+        <v>1.4533</v>
       </c>
       <c r="M3" t="n">
-        <v>1.1671</v>
+        <v>1.1709</v>
       </c>
     </row>
     <row r="4">
@@ -592,25 +592,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C4" t="n">
         <v>34.16</v>
       </c>
       <c r="D4" t="n">
-        <v>19.57</v>
+        <v>19.7</v>
       </c>
       <c r="E4" t="n">
-        <v>5.88</v>
+        <v>5.92</v>
       </c>
       <c r="F4" t="n">
-        <v>19.6108</v>
+        <v>19.7364</v>
       </c>
       <c r="G4" t="n">
         <v>72</v>
       </c>
       <c r="H4" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I4" t="n">
         <v>18</v>
@@ -619,13 +619,13 @@
         <v>18</v>
       </c>
       <c r="K4" t="n">
-        <v>5.67</v>
+        <v>5.69</v>
       </c>
       <c r="L4" t="n">
-        <v>1.4239</v>
+        <v>1.425</v>
       </c>
       <c r="M4" t="n">
-        <v>1.2143</v>
+        <v>1.2201</v>
       </c>
     </row>
     <row r="5">
@@ -635,25 +635,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C5" t="n">
         <v>35.32</v>
       </c>
       <c r="D5" t="n">
-        <v>21.19</v>
+        <v>21.36</v>
       </c>
       <c r="E5" t="n">
-        <v>6.370000000000001</v>
+        <v>6.419999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>21.2336</v>
+        <v>21.4072</v>
       </c>
       <c r="G5" t="n">
         <v>73</v>
       </c>
       <c r="H5" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I5" t="n">
         <v>18</v>
@@ -662,13 +662,13 @@
         <v>17</v>
       </c>
       <c r="K5" t="n">
-        <v>5.76</v>
+        <v>5.66</v>
       </c>
       <c r="L5" t="n">
-        <v>1.4388</v>
+        <v>1.4403</v>
       </c>
       <c r="M5" t="n">
-        <v>1.2019</v>
+        <v>1.198</v>
       </c>
     </row>
     <row r="6">
@@ -678,25 +678,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C6" t="n">
         <v>25.31</v>
       </c>
       <c r="D6" t="n">
-        <v>14.77</v>
+        <v>14.87</v>
       </c>
       <c r="E6" t="n">
-        <v>4.44</v>
+        <v>4.47</v>
       </c>
       <c r="F6" t="n">
-        <v>14.7949</v>
+        <v>14.8981</v>
       </c>
       <c r="G6" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H6" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I6" t="n">
         <v>18</v>
@@ -705,13 +705,13 @@
         <v>18</v>
       </c>
       <c r="K6" t="n">
-        <v>5.01</v>
+        <v>5.04</v>
       </c>
       <c r="L6" t="n">
-        <v>1.3636</v>
+        <v>1.3646</v>
       </c>
       <c r="M6" t="n">
-        <v>1.1939</v>
+        <v>1.2001</v>
       </c>
     </row>
     <row r="7">
@@ -721,25 +721,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C7" t="n">
         <v>36.42</v>
       </c>
       <c r="D7" t="n">
-        <v>22.6</v>
+        <v>22.5</v>
       </c>
       <c r="E7" t="n">
-        <v>6.79</v>
+        <v>6.76</v>
       </c>
       <c r="F7" t="n">
-        <v>22.6418</v>
+        <v>22.5422</v>
       </c>
       <c r="G7" t="n">
         <v>63</v>
       </c>
       <c r="H7" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I7" t="n">
         <v>18</v>
@@ -748,13 +748,13 @@
         <v>18</v>
       </c>
       <c r="K7" t="n">
-        <v>7.48</v>
+        <v>7.47</v>
       </c>
       <c r="L7" t="n">
-        <v>1.4507</v>
+        <v>1.4505</v>
       </c>
       <c r="M7" t="n">
-        <v>1.1589</v>
+        <v>1.1585</v>
       </c>
     </row>
     <row r="8">
@@ -764,25 +764,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C8" t="n">
         <v>32.44</v>
       </c>
       <c r="D8" t="n">
-        <v>20.19</v>
+        <v>20.21</v>
       </c>
       <c r="E8" t="n">
         <v>6.069999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>20.2327</v>
+        <v>20.2483</v>
       </c>
       <c r="G8" t="n">
         <v>70</v>
       </c>
       <c r="H8" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I8" t="n">
         <v>17</v>
@@ -791,13 +791,13 @@
         <v>17</v>
       </c>
       <c r="K8" t="n">
-        <v>5.6</v>
+        <v>5.64</v>
       </c>
       <c r="L8" t="n">
-        <v>1.4312</v>
+        <v>1.431</v>
       </c>
       <c r="M8" t="n">
-        <v>1.1934</v>
+        <v>1.1992</v>
       </c>
     </row>
     <row r="9">
@@ -813,13 +813,13 @@
         <v>36.03</v>
       </c>
       <c r="D9" t="n">
-        <v>22.36</v>
+        <v>22.34</v>
       </c>
       <c r="E9" t="n">
-        <v>6.72</v>
+        <v>6.710000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>22.4085</v>
+        <v>22.3798</v>
       </c>
       <c r="G9" t="n">
         <v>65</v>
@@ -834,13 +834,13 @@
         <v>17</v>
       </c>
       <c r="K9" t="n">
-        <v>7.11</v>
+        <v>7.12</v>
       </c>
       <c r="L9" t="n">
-        <v>1.4509</v>
+        <v>1.4504</v>
       </c>
       <c r="M9" t="n">
-        <v>1.1904</v>
+        <v>1.186</v>
       </c>
     </row>
     <row r="10">
@@ -856,13 +856,13 @@
         <v>34.03</v>
       </c>
       <c r="D10" t="n">
-        <v>21.24</v>
+        <v>21.08</v>
       </c>
       <c r="E10" t="n">
-        <v>6.38</v>
+        <v>6.34</v>
       </c>
       <c r="F10" t="n">
-        <v>21.2784</v>
+        <v>21.1176</v>
       </c>
       <c r="G10" t="n">
         <v>68</v>
@@ -877,13 +877,13 @@
         <v>17</v>
       </c>
       <c r="K10" t="n">
-        <v>5.93</v>
+        <v>5.98</v>
       </c>
       <c r="L10" t="n">
-        <v>1.4405</v>
+        <v>1.4385</v>
       </c>
       <c r="M10" t="n">
-        <v>1.1713</v>
+        <v>1.1728</v>
       </c>
     </row>
   </sheetData>
@@ -974,22 +974,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C2" t="n">
         <v>24.04</v>
       </c>
       <c r="D2" t="n">
-        <v>11.47</v>
+        <v>11.45</v>
       </c>
       <c r="E2" t="n">
-        <v>4.38</v>
+        <v>4.37</v>
       </c>
       <c r="F2" t="n">
-        <v>14.5985</v>
+        <v>14.5749</v>
       </c>
       <c r="G2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H2" t="n">
         <v>52</v>
@@ -1001,13 +1001,13 @@
         <v>18</v>
       </c>
       <c r="K2" t="n">
-        <v>6.19</v>
+        <v>5.94</v>
       </c>
       <c r="L2" t="n">
-        <v>1.2087</v>
+        <v>1.2082</v>
       </c>
       <c r="M2" t="n">
-        <v>1.1885</v>
+        <v>1.1936</v>
       </c>
     </row>
     <row r="3">
@@ -1017,19 +1017,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="C3" t="n">
         <v>34.67</v>
       </c>
       <c r="D3" t="n">
-        <v>130.21</v>
+        <v>130.46</v>
       </c>
       <c r="E3" t="n">
-        <v>6.35</v>
+        <v>6.370000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>21.1816</v>
+        <v>21.2222</v>
       </c>
       <c r="G3" t="n">
         <v>66</v>
@@ -1044,13 +1044,13 @@
         <v>17</v>
       </c>
       <c r="K3" t="n">
-        <v>6.77</v>
+        <v>6.78</v>
       </c>
       <c r="L3" t="n">
-        <v>1.5625</v>
+        <v>1.563</v>
       </c>
       <c r="M3" t="n">
-        <v>1.1688</v>
+        <v>1.1699</v>
       </c>
     </row>
     <row r="4">
@@ -1060,19 +1060,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="C4" t="n">
         <v>32.29</v>
       </c>
       <c r="D4" t="n">
-        <v>60.84</v>
+        <v>61</v>
       </c>
       <c r="E4" t="n">
-        <v>5.850000000000001</v>
+        <v>5.87</v>
       </c>
       <c r="F4" t="n">
-        <v>19.5119</v>
+        <v>19.5619</v>
       </c>
       <c r="G4" t="n">
         <v>67</v>
@@ -1087,13 +1087,13 @@
         <v>17</v>
       </c>
       <c r="K4" t="n">
-        <v>6.66</v>
+        <v>6.7</v>
       </c>
       <c r="L4" t="n">
-        <v>1.5048</v>
+        <v>1.5051</v>
       </c>
       <c r="M4" t="n">
-        <v>1.1628</v>
+        <v>1.1629</v>
       </c>
     </row>
     <row r="5">
@@ -1103,25 +1103,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C5" t="n">
         <v>34.34</v>
       </c>
       <c r="D5" t="n">
-        <v>63.94</v>
+        <v>64.27</v>
       </c>
       <c r="E5" t="n">
-        <v>6.329999999999999</v>
+        <v>6.370000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>21.1075</v>
+        <v>21.2179</v>
       </c>
       <c r="G5" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H5" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I5" t="n">
         <v>17</v>
@@ -1130,13 +1130,13 @@
         <v>17</v>
       </c>
       <c r="K5" t="n">
-        <v>6.55</v>
+        <v>6.5</v>
       </c>
       <c r="L5" t="n">
-        <v>1.5133</v>
+        <v>1.5143</v>
       </c>
       <c r="M5" t="n">
-        <v>1.1827</v>
+        <v>1.1859</v>
       </c>
     </row>
     <row r="6">
@@ -1146,19 +1146,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C6" t="n">
         <v>35.09</v>
       </c>
       <c r="D6" t="n">
-        <v>44.75</v>
+        <v>44.62</v>
       </c>
       <c r="E6" t="n">
-        <v>6.41</v>
+        <v>6.39</v>
       </c>
       <c r="F6" t="n">
-        <v>21.3671</v>
+        <v>21.3056</v>
       </c>
       <c r="G6" t="n">
         <v>64</v>
@@ -1173,13 +1173,13 @@
         <v>17</v>
       </c>
       <c r="K6" t="n">
-        <v>7.15</v>
+        <v>7.13</v>
       </c>
       <c r="L6" t="n">
-        <v>1.4507</v>
+        <v>1.4501</v>
       </c>
       <c r="M6" t="n">
-        <v>1.1632</v>
+        <v>1.1627</v>
       </c>
     </row>
     <row r="7">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C7" t="n">
         <v>33.73</v>
@@ -1201,13 +1201,13 @@
         <v>6.2</v>
       </c>
       <c r="F7" t="n">
-        <v>20.6505</v>
+        <v>20.6507</v>
       </c>
       <c r="G7" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H7" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I7" t="n">
         <v>17</v>
@@ -1216,13 +1216,13 @@
         <v>17</v>
       </c>
       <c r="K7" t="n">
-        <v>5.93</v>
+        <v>5.9</v>
       </c>
       <c r="L7" t="n">
-        <v>1.4472</v>
+        <v>1.4475</v>
       </c>
       <c r="M7" t="n">
-        <v>1.1759</v>
+        <v>1.1775</v>
       </c>
     </row>
     <row r="8">
@@ -1232,19 +1232,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C8" t="n">
         <v>35.28</v>
       </c>
       <c r="D8" t="n">
-        <v>22.84</v>
+        <v>22.8</v>
       </c>
       <c r="E8" t="n">
-        <v>6.54</v>
+        <v>6.529999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>21.8117</v>
+        <v>21.773</v>
       </c>
       <c r="G8" t="n">
         <v>65</v>
@@ -1259,13 +1259,13 @@
         <v>17</v>
       </c>
       <c r="K8" t="n">
-        <v>7.14</v>
+        <v>7.06</v>
       </c>
       <c r="L8" t="n">
-        <v>1.3563</v>
+        <v>1.3558</v>
       </c>
       <c r="M8" t="n">
-        <v>1.1535</v>
+        <v>1.152</v>
       </c>
     </row>
     <row r="9">
@@ -1275,25 +1275,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C9" t="n">
         <v>31.99</v>
       </c>
       <c r="D9" t="n">
-        <v>20.66</v>
+        <v>20.58</v>
       </c>
       <c r="E9" t="n">
-        <v>5.92</v>
+        <v>5.899999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>19.7291</v>
+        <v>19.6516</v>
       </c>
       <c r="G9" t="n">
         <v>67</v>
       </c>
       <c r="H9" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I9" t="n">
         <v>17</v>
@@ -1302,13 +1302,13 @@
         <v>17</v>
       </c>
       <c r="K9" t="n">
-        <v>6.87</v>
+        <v>6.8</v>
       </c>
       <c r="L9" t="n">
-        <v>1.3447</v>
+        <v>1.3437</v>
       </c>
       <c r="M9" t="n">
-        <v>1.2047</v>
+        <v>1.2069</v>
       </c>
     </row>
   </sheetData>
@@ -1399,25 +1399,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C2" t="n">
         <v>30.09</v>
       </c>
       <c r="D2" t="n">
-        <v>14.27</v>
+        <v>14.3</v>
       </c>
       <c r="E2" t="n">
         <v>5.46</v>
       </c>
       <c r="F2" t="n">
-        <v>18.1841</v>
+        <v>18.2163</v>
       </c>
       <c r="G2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I2" t="n">
         <v>17</v>
@@ -1426,13 +1426,13 @@
         <v>17</v>
       </c>
       <c r="K2" t="n">
-        <v>7.43</v>
+        <v>7.27</v>
       </c>
       <c r="L2" t="n">
-        <v>1.3884</v>
+        <v>1.3885</v>
       </c>
       <c r="M2" t="n">
-        <v>1.1514</v>
+        <v>1.1565</v>
       </c>
     </row>
     <row r="3">
@@ -1442,25 +1442,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C3" t="n">
         <v>31.83</v>
       </c>
       <c r="D3" t="n">
-        <v>15.16</v>
+        <v>15.12</v>
       </c>
       <c r="E3" t="n">
-        <v>5.79</v>
+        <v>5.77</v>
       </c>
       <c r="F3" t="n">
-        <v>19.2869</v>
+        <v>19.2357</v>
       </c>
       <c r="G3" t="n">
         <v>68</v>
       </c>
       <c r="H3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I3" t="n">
         <v>17</v>
@@ -1469,13 +1469,13 @@
         <v>17</v>
       </c>
       <c r="K3" t="n">
-        <v>6.46</v>
+        <v>6.42</v>
       </c>
       <c r="L3" t="n">
-        <v>1.399</v>
+        <v>1.3982</v>
       </c>
       <c r="M3" t="n">
-        <v>1.1545</v>
+        <v>1.1535</v>
       </c>
     </row>
     <row r="4">
@@ -1485,22 +1485,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C4" t="n">
         <v>34.14</v>
       </c>
       <c r="D4" t="n">
-        <v>16.21</v>
+        <v>16.23</v>
       </c>
       <c r="E4" t="n">
-        <v>6.21</v>
+        <v>6.22</v>
       </c>
       <c r="F4" t="n">
-        <v>20.6909</v>
+        <v>20.7181</v>
       </c>
       <c r="G4" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H4" t="n">
         <v>46</v>
@@ -1512,13 +1512,13 @@
         <v>17</v>
       </c>
       <c r="K4" t="n">
-        <v>6.6</v>
+        <v>6.47</v>
       </c>
       <c r="L4" t="n">
-        <v>1.3752</v>
+        <v>1.3751</v>
       </c>
       <c r="M4" t="n">
-        <v>1.1665</v>
+        <v>1.1694</v>
       </c>
     </row>
     <row r="5">
@@ -1528,22 +1528,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C5" t="n">
         <v>29.49</v>
       </c>
       <c r="D5" t="n">
-        <v>13.51</v>
+        <v>13.5</v>
       </c>
       <c r="E5" t="n">
-        <v>5.31</v>
+        <v>5.3</v>
       </c>
       <c r="F5" t="n">
-        <v>17.6885</v>
+        <v>17.6773</v>
       </c>
       <c r="G5" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H5" t="n">
         <v>58</v>
@@ -1555,13 +1555,13 @@
         <v>17</v>
       </c>
       <c r="K5" t="n">
-        <v>5.33</v>
+        <v>5.41</v>
       </c>
       <c r="L5" t="n">
-        <v>1.3819</v>
+        <v>1.3814</v>
       </c>
       <c r="M5" t="n">
-        <v>1.2064</v>
+        <v>1.2075</v>
       </c>
     </row>
     <row r="6">
@@ -1577,19 +1577,19 @@
         <v>33.07</v>
       </c>
       <c r="D6" t="n">
-        <v>15.58</v>
+        <v>15.71</v>
       </c>
       <c r="E6" t="n">
-        <v>6.12</v>
+        <v>6.17</v>
       </c>
       <c r="F6" t="n">
-        <v>20.3906</v>
+        <v>20.5525</v>
       </c>
       <c r="G6" t="n">
         <v>69</v>
       </c>
       <c r="H6" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I6" t="n">
         <v>16</v>
@@ -1598,13 +1598,13 @@
         <v>17</v>
       </c>
       <c r="K6" t="n">
-        <v>5.58</v>
+        <v>5.54</v>
       </c>
       <c r="L6" t="n">
-        <v>1.3995</v>
+        <v>1.4009</v>
       </c>
       <c r="M6" t="n">
-        <v>1.1856</v>
+        <v>1.1842</v>
       </c>
     </row>
     <row r="7">
@@ -1614,25 +1614,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C7" t="n">
         <v>33.61</v>
       </c>
       <c r="D7" t="n">
-        <v>15.35</v>
+        <v>15.12</v>
       </c>
       <c r="E7" t="n">
-        <v>6.239999999999999</v>
+        <v>6.140000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>20.7848</v>
+        <v>20.4766</v>
       </c>
       <c r="G7" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H7" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I7" t="n">
         <v>17</v>
@@ -1641,13 +1641,13 @@
         <v>17</v>
       </c>
       <c r="K7" t="n">
-        <v>6.38</v>
+        <v>6.35</v>
       </c>
       <c r="L7" t="n">
-        <v>1.4015</v>
+        <v>1.3987</v>
       </c>
       <c r="M7" t="n">
-        <v>1.1795</v>
+        <v>1.1826</v>
       </c>
     </row>
     <row r="8">
@@ -1657,22 +1657,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C8" t="n">
         <v>31.81</v>
       </c>
       <c r="D8" t="n">
-        <v>14.66</v>
+        <v>14.67</v>
       </c>
       <c r="E8" t="n">
-        <v>5.93</v>
+        <v>5.94</v>
       </c>
       <c r="F8" t="n">
-        <v>19.7807</v>
+        <v>19.7964</v>
       </c>
       <c r="G8" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H8" t="n">
         <v>54</v>
@@ -1684,13 +1684,13 @@
         <v>17</v>
       </c>
       <c r="K8" t="n">
-        <v>6.55</v>
+        <v>6.61</v>
       </c>
       <c r="L8" t="n">
-        <v>1.3924</v>
+        <v>1.3925</v>
       </c>
       <c r="M8" t="n">
-        <v>1.1902</v>
+        <v>1.1989</v>
       </c>
     </row>
     <row r="9">
@@ -1706,13 +1706,13 @@
         <v>35.48</v>
       </c>
       <c r="D9" t="n">
-        <v>16.99</v>
+        <v>16.94</v>
       </c>
       <c r="E9" t="n">
-        <v>6.49</v>
+        <v>6.47</v>
       </c>
       <c r="F9" t="n">
-        <v>21.6355</v>
+        <v>21.5717</v>
       </c>
       <c r="G9" t="n">
         <v>64</v>
@@ -1727,13 +1727,13 @@
         <v>17</v>
       </c>
       <c r="K9" t="n">
-        <v>6.77</v>
+        <v>6.79</v>
       </c>
       <c r="L9" t="n">
-        <v>1.3834</v>
+        <v>1.3838</v>
       </c>
       <c r="M9" t="n">
-        <v>1.1776</v>
+        <v>1.1793</v>
       </c>
     </row>
     <row r="10">
@@ -1743,25 +1743,25 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C10" t="n">
         <v>35.56</v>
       </c>
       <c r="D10" t="n">
-        <v>34.14</v>
+        <v>34.06</v>
       </c>
       <c r="E10" t="n">
-        <v>6.52</v>
+        <v>6.510000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>21.7411</v>
+        <v>21.6902</v>
       </c>
       <c r="G10" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H10" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I10" t="n">
         <v>17</v>
@@ -1770,13 +1770,13 @@
         <v>17</v>
       </c>
       <c r="K10" t="n">
-        <v>7.29</v>
+        <v>7.37</v>
       </c>
       <c r="L10" t="n">
-        <v>1.4134</v>
+        <v>1.4135</v>
       </c>
       <c r="M10" t="n">
-        <v>1.1632</v>
+        <v>1.1585</v>
       </c>
     </row>
     <row r="11">
@@ -1786,19 +1786,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C11" t="n">
         <v>33.94</v>
       </c>
       <c r="D11" t="n">
-        <v>31.77</v>
+        <v>31.78</v>
       </c>
       <c r="E11" t="n">
         <v>6.239999999999999</v>
       </c>
       <c r="F11" t="n">
-        <v>20.7917</v>
+        <v>20.7966</v>
       </c>
       <c r="G11" t="n">
         <v>70</v>
@@ -1813,13 +1813,13 @@
         <v>17</v>
       </c>
       <c r="K11" t="n">
-        <v>5.76</v>
+        <v>5.79</v>
       </c>
       <c r="L11" t="n">
-        <v>1.4133</v>
+        <v>1.4136</v>
       </c>
       <c r="M11" t="n">
-        <v>1.1863</v>
+        <v>1.1844</v>
       </c>
     </row>
   </sheetData>
@@ -1910,19 +1910,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C2" t="n">
         <v>24.04</v>
       </c>
       <c r="D2" t="n">
-        <v>11.43</v>
+        <v>11.42</v>
       </c>
       <c r="E2" t="n">
-        <v>4.37</v>
+        <v>4.36</v>
       </c>
       <c r="F2" t="n">
-        <v>14.5558</v>
+        <v>14.5394</v>
       </c>
       <c r="G2" t="n">
         <v>71</v>
@@ -1937,13 +1937,13 @@
         <v>18</v>
       </c>
       <c r="K2" t="n">
-        <v>6.12</v>
+        <v>6.04</v>
       </c>
       <c r="L2" t="n">
-        <v>1.2077</v>
+        <v>1.2076</v>
       </c>
       <c r="M2" t="n">
-        <v>1.2024</v>
+        <v>1.1964</v>
       </c>
     </row>
     <row r="3">
@@ -1953,19 +1953,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="C3" t="n">
         <v>36.62</v>
       </c>
       <c r="D3" t="n">
-        <v>53.1</v>
+        <v>52.95</v>
       </c>
       <c r="E3" t="n">
-        <v>6.76</v>
+        <v>6.74</v>
       </c>
       <c r="F3" t="n">
-        <v>22.5332</v>
+        <v>22.4721</v>
       </c>
       <c r="G3" t="n">
         <v>66</v>
@@ -1980,13 +1980,13 @@
         <v>17</v>
       </c>
       <c r="K3" t="n">
-        <v>7.06</v>
+        <v>7.01</v>
       </c>
       <c r="L3" t="n">
-        <v>1.4235</v>
+        <v>1.423</v>
       </c>
       <c r="M3" t="n">
-        <v>1.1595</v>
+        <v>1.1583</v>
       </c>
     </row>
     <row r="4">
@@ -1996,25 +1996,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="C4" t="n">
         <v>33.46</v>
       </c>
       <c r="D4" t="n">
-        <v>77.29000000000001</v>
+        <v>77.48</v>
       </c>
       <c r="E4" t="n">
-        <v>6.12</v>
+        <v>6.13</v>
       </c>
       <c r="F4" t="n">
-        <v>20.3873</v>
+        <v>20.4377</v>
       </c>
       <c r="G4" t="n">
         <v>68</v>
       </c>
       <c r="H4" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I4" t="n">
         <v>17</v>
@@ -2023,13 +2023,13 @@
         <v>17</v>
       </c>
       <c r="K4" t="n">
-        <v>6.09</v>
+        <v>6.14</v>
       </c>
       <c r="L4" t="n">
-        <v>1.475</v>
+        <v>1.4753</v>
       </c>
       <c r="M4" t="n">
-        <v>1.1844</v>
+        <v>1.1846</v>
       </c>
     </row>
   </sheetData>
@@ -2126,16 +2126,16 @@
         <v>31.71</v>
       </c>
       <c r="D2" t="n">
-        <v>15.76</v>
+        <v>15.75</v>
       </c>
       <c r="E2" t="n">
-        <v>5.800000000000001</v>
+        <v>5.79</v>
       </c>
       <c r="F2" t="n">
-        <v>19.333</v>
+        <v>19.3136</v>
       </c>
       <c r="G2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H2" t="n">
         <v>53</v>
@@ -2150,10 +2150,10 @@
         <v>6.41</v>
       </c>
       <c r="L2" t="n">
-        <v>1.4078</v>
+        <v>1.4073</v>
       </c>
       <c r="M2" t="n">
-        <v>1.1744</v>
+        <v>1.1784</v>
       </c>
     </row>
     <row r="3">
@@ -2169,13 +2169,13 @@
         <v>32.89</v>
       </c>
       <c r="D3" t="n">
-        <v>17.01</v>
+        <v>16.91</v>
       </c>
       <c r="E3" t="n">
-        <v>5.850000000000001</v>
+        <v>5.81</v>
       </c>
       <c r="F3" t="n">
-        <v>19.486</v>
+        <v>19.3767</v>
       </c>
       <c r="G3" t="n">
         <v>72</v>
@@ -2190,13 +2190,13 @@
         <v>18</v>
       </c>
       <c r="K3" t="n">
-        <v>5.64</v>
+        <v>5.68</v>
       </c>
       <c r="L3" t="n">
-        <v>1.4213</v>
+        <v>1.4203</v>
       </c>
       <c r="M3" t="n">
-        <v>1.1924</v>
+        <v>1.1884</v>
       </c>
     </row>
     <row r="4">
@@ -2206,22 +2206,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C4" t="n">
         <v>34.04</v>
       </c>
       <c r="D4" t="n">
-        <v>17.85</v>
+        <v>17.93</v>
       </c>
       <c r="E4" t="n">
-        <v>6.15</v>
+        <v>6.18</v>
       </c>
       <c r="F4" t="n">
-        <v>20.498</v>
+        <v>20.59</v>
       </c>
       <c r="G4" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H4" t="n">
         <v>49</v>
@@ -2233,13 +2233,13 @@
         <v>17</v>
       </c>
       <c r="K4" t="n">
-        <v>5.88</v>
+        <v>5.97</v>
       </c>
       <c r="L4" t="n">
         <v>1.4048</v>
       </c>
       <c r="M4" t="n">
-        <v>1.1743</v>
+        <v>1.1719</v>
       </c>
     </row>
     <row r="5">
@@ -2255,19 +2255,19 @@
         <v>32.02999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>11.59</v>
+        <v>11.6</v>
       </c>
       <c r="E5" t="n">
-        <v>5.53</v>
+        <v>5.54</v>
       </c>
       <c r="F5" t="n">
-        <v>18.4348</v>
+        <v>18.4547</v>
       </c>
       <c r="G5" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H5" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I5" t="n">
         <v>19</v>
@@ -2276,13 +2276,13 @@
         <v>18</v>
       </c>
       <c r="K5" t="n">
-        <v>5.18</v>
+        <v>5.17</v>
       </c>
       <c r="L5" t="n">
-        <v>1.3848</v>
+        <v>1.3833</v>
       </c>
       <c r="M5" t="n">
-        <v>1.2841</v>
+        <v>1.2838</v>
       </c>
     </row>
     <row r="6">
@@ -2298,16 +2298,16 @@
         <v>32.88</v>
       </c>
       <c r="D6" t="n">
-        <v>12.62</v>
+        <v>12.58</v>
       </c>
       <c r="E6" t="n">
-        <v>6.03</v>
+        <v>6.02</v>
       </c>
       <c r="F6" t="n">
-        <v>20.1128</v>
+        <v>20.0559</v>
       </c>
       <c r="G6" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H6" t="n">
         <v>57</v>
@@ -2319,13 +2319,13 @@
         <v>17</v>
       </c>
       <c r="K6" t="n">
-        <v>4.99</v>
+        <v>5.01</v>
       </c>
       <c r="L6" t="n">
-        <v>1.3895</v>
+        <v>1.3892</v>
       </c>
       <c r="M6" t="n">
-        <v>1.2136</v>
+        <v>1.2131</v>
       </c>
     </row>
     <row r="7">
@@ -2335,25 +2335,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C7" t="n">
         <v>32.71</v>
       </c>
       <c r="D7" t="n">
-        <v>11.42</v>
+        <v>11.44</v>
       </c>
       <c r="E7" t="n">
-        <v>6.09</v>
+        <v>6.1</v>
       </c>
       <c r="F7" t="n">
-        <v>20.3148</v>
+        <v>20.3425</v>
       </c>
       <c r="G7" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H7" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I7" t="n">
         <v>18</v>
@@ -2362,13 +2362,13 @@
         <v>17</v>
       </c>
       <c r="K7" t="n">
-        <v>5.78</v>
+        <v>5.86</v>
       </c>
       <c r="L7" t="n">
-        <v>1.3756</v>
+        <v>1.3755</v>
       </c>
       <c r="M7" t="n">
-        <v>1.186</v>
+        <v>1.202</v>
       </c>
     </row>
     <row r="8">
@@ -2384,19 +2384,19 @@
         <v>32.76</v>
       </c>
       <c r="D8" t="n">
-        <v>11.46</v>
+        <v>11.5</v>
       </c>
       <c r="E8" t="n">
-        <v>6.1</v>
+        <v>6.12</v>
       </c>
       <c r="F8" t="n">
-        <v>20.3365</v>
+        <v>20.4076</v>
       </c>
       <c r="G8" t="n">
         <v>70</v>
       </c>
       <c r="H8" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I8" t="n">
         <v>18</v>
@@ -2405,13 +2405,13 @@
         <v>17</v>
       </c>
       <c r="K8" t="n">
-        <v>6.2</v>
+        <v>6.17</v>
       </c>
       <c r="L8" t="n">
-        <v>1.3773</v>
+        <v>1.378</v>
       </c>
       <c r="M8" t="n">
-        <v>1.1892</v>
+        <v>1.1872</v>
       </c>
     </row>
     <row r="9">
@@ -2427,19 +2427,19 @@
         <v>33.06</v>
       </c>
       <c r="D9" t="n">
-        <v>16.17</v>
+        <v>16.15</v>
       </c>
       <c r="E9" t="n">
-        <v>5.96</v>
+        <v>5.949999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>19.8543</v>
+        <v>19.8347</v>
       </c>
       <c r="G9" t="n">
         <v>67</v>
       </c>
       <c r="H9" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I9" t="n">
         <v>17</v>
@@ -2448,13 +2448,13 @@
         <v>17</v>
       </c>
       <c r="K9" t="n">
-        <v>6</v>
+        <v>6.01</v>
       </c>
       <c r="L9" t="n">
-        <v>1.3832</v>
+        <v>1.3831</v>
       </c>
       <c r="M9" t="n">
-        <v>1.1855</v>
+        <v>1.1808</v>
       </c>
     </row>
     <row r="10">
@@ -2464,25 +2464,25 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="C10" t="n">
         <v>33.2</v>
       </c>
       <c r="D10" t="n">
-        <v>62.8</v>
+        <v>62.91</v>
       </c>
       <c r="E10" t="n">
-        <v>5.91</v>
+        <v>5.92</v>
       </c>
       <c r="F10" t="n">
-        <v>19.7003</v>
+        <v>19.7359</v>
       </c>
       <c r="G10" t="n">
         <v>69</v>
       </c>
       <c r="H10" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I10" t="n">
         <v>18</v>
@@ -2491,13 +2491,13 @@
         <v>17</v>
       </c>
       <c r="K10" t="n">
-        <v>5.94</v>
+        <v>5.99</v>
       </c>
       <c r="L10" t="n">
-        <v>1.5138</v>
+        <v>1.5142</v>
       </c>
       <c r="M10" t="n">
-        <v>1.1929</v>
+        <v>1.1928</v>
       </c>
     </row>
     <row r="11">
@@ -2513,13 +2513,13 @@
         <v>33.27</v>
       </c>
       <c r="D11" t="n">
-        <v>52.42</v>
+        <v>52.51</v>
       </c>
       <c r="E11" t="n">
-        <v>6.13</v>
+        <v>6.140000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>20.4176</v>
+        <v>20.4516</v>
       </c>
       <c r="G11" t="n">
         <v>71</v>
@@ -2534,13 +2534,13 @@
         <v>17</v>
       </c>
       <c r="K11" t="n">
-        <v>5.86</v>
+        <v>5.85</v>
       </c>
       <c r="L11" t="n">
-        <v>1.4861</v>
+        <v>1.4862</v>
       </c>
       <c r="M11" t="n">
-        <v>1.1942</v>
+        <v>1.1932</v>
       </c>
     </row>
     <row r="12">
@@ -2550,25 +2550,25 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C12" t="n">
         <v>34.32</v>
       </c>
       <c r="D12" t="n">
-        <v>35.71</v>
+        <v>35.72</v>
       </c>
       <c r="E12" t="n">
-        <v>6.140000000000001</v>
+        <v>6.15</v>
       </c>
       <c r="F12" t="n">
-        <v>20.482</v>
+        <v>20.4884</v>
       </c>
       <c r="G12" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H12" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I12" t="n">
         <v>18</v>
@@ -2577,13 +2577,13 @@
         <v>17</v>
       </c>
       <c r="K12" t="n">
-        <v>5.68</v>
+        <v>5.8</v>
       </c>
       <c r="L12" t="n">
-        <v>1.4243</v>
+        <v>1.4241</v>
       </c>
       <c r="M12" t="n">
-        <v>1.1798</v>
+        <v>1.178</v>
       </c>
     </row>
     <row r="13">
@@ -2593,25 +2593,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C13" t="n">
         <v>33.65000000000001</v>
       </c>
       <c r="D13" t="n">
-        <v>23.64</v>
+        <v>23.59</v>
       </c>
       <c r="E13" t="n">
-        <v>6.3</v>
+        <v>6.279999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>20.9973</v>
+        <v>20.949</v>
       </c>
       <c r="G13" t="n">
         <v>69</v>
       </c>
       <c r="H13" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I13" t="n">
         <v>18</v>
@@ -2620,13 +2620,13 @@
         <v>17</v>
       </c>
       <c r="K13" t="n">
-        <v>6.13</v>
+        <v>6.1</v>
       </c>
       <c r="L13" t="n">
-        <v>1.375</v>
+        <v>1.3747</v>
       </c>
       <c r="M13" t="n">
-        <v>1.1894</v>
+        <v>1.1921</v>
       </c>
     </row>
     <row r="14">
@@ -2636,7 +2636,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C14" t="n">
         <v>34.03</v>
@@ -2648,13 +2648,13 @@
         <v>6.08</v>
       </c>
       <c r="F14" t="n">
-        <v>20.2652</v>
+        <v>20.2665</v>
       </c>
       <c r="G14" t="n">
         <v>72</v>
       </c>
       <c r="H14" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I14" t="n">
         <v>18</v>
@@ -2663,13 +2663,13 @@
         <v>17</v>
       </c>
       <c r="K14" t="n">
-        <v>5.26</v>
+        <v>5.38</v>
       </c>
       <c r="L14" t="n">
-        <v>1.3921</v>
+        <v>1.3915</v>
       </c>
       <c r="M14" t="n">
-        <v>1.2386</v>
+        <v>1.2394</v>
       </c>
     </row>
     <row r="15">
@@ -2679,25 +2679,25 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C15" t="n">
         <v>33.93</v>
       </c>
       <c r="D15" t="n">
-        <v>33.55</v>
+        <v>33.38</v>
       </c>
       <c r="E15" t="n">
-        <v>6.18</v>
+        <v>6.140000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>20.5903</v>
+        <v>20.4816</v>
       </c>
       <c r="G15" t="n">
         <v>66</v>
       </c>
       <c r="H15" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I15" t="n">
         <v>18</v>
@@ -2706,13 +2706,13 @@
         <v>17</v>
       </c>
       <c r="K15" t="n">
-        <v>6.35</v>
+        <v>6.32</v>
       </c>
       <c r="L15" t="n">
-        <v>1.4134</v>
+        <v>1.412</v>
       </c>
       <c r="M15" t="n">
-        <v>1.1764</v>
+        <v>1.176</v>
       </c>
     </row>
     <row r="16">
@@ -2722,25 +2722,25 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="C16" t="n">
         <v>34.01</v>
       </c>
       <c r="D16" t="n">
-        <v>118.07</v>
+        <v>118.31</v>
       </c>
       <c r="E16" t="n">
-        <v>6.15</v>
+        <v>6.17</v>
       </c>
       <c r="F16" t="n">
-        <v>20.5161</v>
+        <v>20.5568</v>
       </c>
       <c r="G16" t="n">
         <v>70</v>
       </c>
       <c r="H16" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I16" t="n">
         <v>18</v>
@@ -2755,7 +2755,7 @@
         <v>1.5506</v>
       </c>
       <c r="M16" t="n">
-        <v>1.1892</v>
+        <v>1.1928</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update test for regional analysis
</commit_message>
<xml_diff>
--- a/individual image/first-image/5000/5000 - Regional Analysis.xlsx
+++ b/individual image/first-image/5000/5000 - Regional Analysis.xlsx
@@ -9,9 +9,9 @@
   <sheets>
     <sheet name="Regional analysis_Square grid" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Regional analysis_ETDRS grid" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Regional analysis_Extended ETDR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Regional analysis_Extended" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Regional analysis_Foveal rings" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Regional analysis_Optic nerve h" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Regional analysis_ONH" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -506,25 +506,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C2" t="n">
         <v>33.92</v>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>20.09</v>
       </c>
       <c r="E2" t="n">
-        <v>6.01</v>
+        <v>6.04</v>
       </c>
       <c r="F2" t="n">
-        <v>20.0369</v>
+        <v>20.1298</v>
       </c>
       <c r="G2" t="n">
         <v>70</v>
       </c>
       <c r="H2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I2" t="n">
         <v>19</v>
@@ -533,13 +533,13 @@
         <v>18</v>
       </c>
       <c r="K2" t="n">
-        <v>5.65</v>
+        <v>5.67</v>
       </c>
       <c r="L2" t="n">
-        <v>1.4298</v>
+        <v>1.4291</v>
       </c>
       <c r="M2" t="n">
-        <v>1.2134</v>
+        <v>1.2151</v>
       </c>
     </row>
     <row r="3">
@@ -549,25 +549,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C3" t="n">
         <v>36.44</v>
       </c>
       <c r="D3" t="n">
-        <v>22.84</v>
+        <v>22.81</v>
       </c>
       <c r="E3" t="n">
-        <v>6.87</v>
+        <v>6.859999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>22.8844</v>
+        <v>22.8565</v>
       </c>
       <c r="G3" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H3" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I3" t="n">
         <v>17</v>
@@ -576,13 +576,13 @@
         <v>17</v>
       </c>
       <c r="K3" t="n">
-        <v>6.87</v>
+        <v>7.01</v>
       </c>
       <c r="L3" t="n">
-        <v>1.4533</v>
+        <v>1.4542</v>
       </c>
       <c r="M3" t="n">
-        <v>1.1709</v>
+        <v>1.1651</v>
       </c>
     </row>
     <row r="4">
@@ -592,40 +592,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C4" t="n">
         <v>34.16</v>
       </c>
       <c r="D4" t="n">
-        <v>19.7</v>
+        <v>19.43</v>
       </c>
       <c r="E4" t="n">
-        <v>5.92</v>
+        <v>5.84</v>
       </c>
       <c r="F4" t="n">
-        <v>19.7364</v>
+        <v>19.4721</v>
       </c>
       <c r="G4" t="n">
         <v>72</v>
       </c>
       <c r="H4" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J4" t="n">
         <v>18</v>
       </c>
       <c r="K4" t="n">
-        <v>5.69</v>
+        <v>5.56</v>
       </c>
       <c r="L4" t="n">
-        <v>1.425</v>
+        <v>1.4219</v>
       </c>
       <c r="M4" t="n">
-        <v>1.2201</v>
+        <v>1.2001</v>
       </c>
     </row>
     <row r="5">
@@ -635,22 +635,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C5" t="n">
         <v>35.32</v>
       </c>
       <c r="D5" t="n">
-        <v>21.36</v>
+        <v>21.16</v>
       </c>
       <c r="E5" t="n">
-        <v>6.419999999999999</v>
+        <v>6.36</v>
       </c>
       <c r="F5" t="n">
-        <v>21.4072</v>
+        <v>21.2034</v>
       </c>
       <c r="G5" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H5" t="n">
         <v>57</v>
@@ -662,13 +662,13 @@
         <v>17</v>
       </c>
       <c r="K5" t="n">
-        <v>5.66</v>
+        <v>5.77</v>
       </c>
       <c r="L5" t="n">
-        <v>1.4403</v>
+        <v>1.4392</v>
       </c>
       <c r="M5" t="n">
-        <v>1.198</v>
+        <v>1.1936</v>
       </c>
     </row>
     <row r="6">
@@ -684,13 +684,13 @@
         <v>25.31</v>
       </c>
       <c r="D6" t="n">
-        <v>14.87</v>
+        <v>14.93</v>
       </c>
       <c r="E6" t="n">
-        <v>4.47</v>
+        <v>4.49</v>
       </c>
       <c r="F6" t="n">
-        <v>14.8981</v>
+        <v>14.9586</v>
       </c>
       <c r="G6" t="n">
         <v>80</v>
@@ -705,13 +705,13 @@
         <v>18</v>
       </c>
       <c r="K6" t="n">
-        <v>5.04</v>
+        <v>5.02</v>
       </c>
       <c r="L6" t="n">
-        <v>1.3646</v>
+        <v>1.365</v>
       </c>
       <c r="M6" t="n">
-        <v>1.2001</v>
+        <v>1.2047</v>
       </c>
     </row>
     <row r="7">
@@ -721,25 +721,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C7" t="n">
         <v>36.42</v>
       </c>
       <c r="D7" t="n">
-        <v>22.5</v>
+        <v>22.56</v>
       </c>
       <c r="E7" t="n">
-        <v>6.76</v>
+        <v>6.78</v>
       </c>
       <c r="F7" t="n">
-        <v>22.5422</v>
+        <v>22.6029</v>
       </c>
       <c r="G7" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H7" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I7" t="n">
         <v>18</v>
@@ -748,13 +748,13 @@
         <v>18</v>
       </c>
       <c r="K7" t="n">
-        <v>7.47</v>
+        <v>7.54</v>
       </c>
       <c r="L7" t="n">
-        <v>1.4505</v>
+        <v>1.4501</v>
       </c>
       <c r="M7" t="n">
-        <v>1.1585</v>
+        <v>1.1583</v>
       </c>
     </row>
     <row r="8">
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C8" t="n">
         <v>32.44</v>
@@ -773,16 +773,16 @@
         <v>20.21</v>
       </c>
       <c r="E8" t="n">
-        <v>6.069999999999999</v>
+        <v>6.08</v>
       </c>
       <c r="F8" t="n">
-        <v>20.2483</v>
+        <v>20.2527</v>
       </c>
       <c r="G8" t="n">
         <v>70</v>
       </c>
       <c r="H8" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I8" t="n">
         <v>17</v>
@@ -791,13 +791,13 @@
         <v>17</v>
       </c>
       <c r="K8" t="n">
-        <v>5.64</v>
+        <v>5.59</v>
       </c>
       <c r="L8" t="n">
-        <v>1.431</v>
+        <v>1.4308</v>
       </c>
       <c r="M8" t="n">
-        <v>1.1992</v>
+        <v>1.1996</v>
       </c>
     </row>
     <row r="9">
@@ -807,25 +807,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C9" t="n">
         <v>36.03</v>
       </c>
       <c r="D9" t="n">
-        <v>22.34</v>
+        <v>22.37</v>
       </c>
       <c r="E9" t="n">
-        <v>6.710000000000001</v>
+        <v>6.73</v>
       </c>
       <c r="F9" t="n">
-        <v>22.3798</v>
+        <v>22.4175</v>
       </c>
       <c r="G9" t="n">
         <v>65</v>
       </c>
       <c r="H9" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I9" t="n">
         <v>17</v>
@@ -834,10 +834,10 @@
         <v>17</v>
       </c>
       <c r="K9" t="n">
-        <v>7.12</v>
+        <v>7.15</v>
       </c>
       <c r="L9" t="n">
-        <v>1.4504</v>
+        <v>1.4501</v>
       </c>
       <c r="M9" t="n">
         <v>1.186</v>
@@ -850,25 +850,25 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C10" t="n">
         <v>34.03</v>
       </c>
       <c r="D10" t="n">
-        <v>21.08</v>
+        <v>21.19</v>
       </c>
       <c r="E10" t="n">
-        <v>6.34</v>
+        <v>6.370000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>21.1176</v>
+        <v>21.2322</v>
       </c>
       <c r="G10" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H10" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I10" t="n">
         <v>18</v>
@@ -877,13 +877,13 @@
         <v>17</v>
       </c>
       <c r="K10" t="n">
-        <v>5.98</v>
+        <v>6.09</v>
       </c>
       <c r="L10" t="n">
-        <v>1.4385</v>
+        <v>1.4396</v>
       </c>
       <c r="M10" t="n">
-        <v>1.1728</v>
+        <v>1.1697</v>
       </c>
     </row>
   </sheetData>
@@ -974,40 +974,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="C2" t="n">
-        <v>24.04</v>
+        <v>22.01</v>
       </c>
       <c r="D2" t="n">
-        <v>11.45</v>
+        <v>9.98</v>
       </c>
       <c r="E2" t="n">
-        <v>4.37</v>
+        <v>3.81</v>
       </c>
       <c r="F2" t="n">
-        <v>14.5749</v>
+        <v>12.7126</v>
       </c>
       <c r="G2" t="n">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="H2" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="I2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J2" t="n">
         <v>18</v>
       </c>
       <c r="K2" t="n">
-        <v>5.94</v>
+        <v>4.51</v>
       </c>
       <c r="L2" t="n">
-        <v>1.2082</v>
+        <v>1.1817</v>
       </c>
       <c r="M2" t="n">
-        <v>1.1936</v>
+        <v>1.1449</v>
       </c>
     </row>
     <row r="3">
@@ -1017,19 +1017,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>885</v>
+        <v>910</v>
       </c>
       <c r="C3" t="n">
-        <v>34.67</v>
+        <v>35.07</v>
       </c>
       <c r="D3" t="n">
-        <v>130.46</v>
+        <v>132.28</v>
       </c>
       <c r="E3" t="n">
-        <v>6.370000000000001</v>
+        <v>6.460000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>21.2222</v>
+        <v>21.5182</v>
       </c>
       <c r="G3" t="n">
         <v>66</v>
@@ -1044,13 +1044,13 @@
         <v>17</v>
       </c>
       <c r="K3" t="n">
-        <v>6.78</v>
+        <v>6.88</v>
       </c>
       <c r="L3" t="n">
-        <v>1.563</v>
+        <v>1.5655</v>
       </c>
       <c r="M3" t="n">
-        <v>1.1699</v>
+        <v>1.1716</v>
       </c>
     </row>
     <row r="4">
@@ -1060,25 +1060,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>409</v>
+        <v>434</v>
       </c>
       <c r="C4" t="n">
-        <v>32.29</v>
+        <v>34.9</v>
       </c>
       <c r="D4" t="n">
-        <v>61</v>
+        <v>64.98</v>
       </c>
       <c r="E4" t="n">
-        <v>5.87</v>
+        <v>6.39</v>
       </c>
       <c r="F4" t="n">
-        <v>19.5619</v>
+        <v>21.3033</v>
       </c>
       <c r="G4" t="n">
         <v>67</v>
       </c>
       <c r="H4" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I4" t="n">
         <v>17</v>
@@ -1087,13 +1087,13 @@
         <v>17</v>
       </c>
       <c r="K4" t="n">
-        <v>6.7</v>
+        <v>6.68</v>
       </c>
       <c r="L4" t="n">
-        <v>1.5051</v>
+        <v>1.5157</v>
       </c>
       <c r="M4" t="n">
-        <v>1.1629</v>
+        <v>1.1668</v>
       </c>
     </row>
     <row r="5">
@@ -1103,25 +1103,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>418</v>
+        <v>450</v>
       </c>
       <c r="C5" t="n">
-        <v>34.34</v>
+        <v>33.77</v>
       </c>
       <c r="D5" t="n">
-        <v>64.27</v>
+        <v>64.53</v>
       </c>
       <c r="E5" t="n">
-        <v>6.370000000000001</v>
+        <v>6.25</v>
       </c>
       <c r="F5" t="n">
-        <v>21.2179</v>
+        <v>20.8355</v>
       </c>
       <c r="G5" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H5" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I5" t="n">
         <v>17</v>
@@ -1130,13 +1130,13 @@
         <v>17</v>
       </c>
       <c r="K5" t="n">
-        <v>6.5</v>
+        <v>6.97</v>
       </c>
       <c r="L5" t="n">
-        <v>1.5143</v>
+        <v>1.5152</v>
       </c>
       <c r="M5" t="n">
-        <v>1.1859</v>
+        <v>1.1821</v>
       </c>
     </row>
     <row r="6">
@@ -1146,22 +1146,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>318</v>
+        <v>309</v>
       </c>
       <c r="C6" t="n">
-        <v>35.09</v>
+        <v>34.97</v>
       </c>
       <c r="D6" t="n">
-        <v>44.62</v>
+        <v>43.04</v>
       </c>
       <c r="E6" t="n">
-        <v>6.39</v>
+        <v>6.45</v>
       </c>
       <c r="F6" t="n">
-        <v>21.3056</v>
+        <v>21.5032</v>
       </c>
       <c r="G6" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H6" t="n">
         <v>51</v>
@@ -1173,13 +1173,13 @@
         <v>17</v>
       </c>
       <c r="K6" t="n">
-        <v>7.13</v>
+        <v>7.18</v>
       </c>
       <c r="L6" t="n">
-        <v>1.4501</v>
+        <v>1.4461</v>
       </c>
       <c r="M6" t="n">
-        <v>1.1627</v>
+        <v>1.1654</v>
       </c>
     </row>
     <row r="7">
@@ -1189,25 +1189,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>250</v>
+        <v>271</v>
       </c>
       <c r="C7" t="n">
-        <v>33.73</v>
+        <v>34.28</v>
       </c>
       <c r="D7" t="n">
-        <v>42.36</v>
+        <v>43.99</v>
       </c>
       <c r="E7" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="F7" t="n">
-        <v>20.6507</v>
+        <v>21.0003</v>
       </c>
       <c r="G7" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H7" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I7" t="n">
         <v>17</v>
@@ -1216,13 +1216,13 @@
         <v>17</v>
       </c>
       <c r="K7" t="n">
-        <v>5.9</v>
+        <v>6.16</v>
       </c>
       <c r="L7" t="n">
-        <v>1.4475</v>
+        <v>1.4488</v>
       </c>
       <c r="M7" t="n">
-        <v>1.1775</v>
+        <v>1.1852</v>
       </c>
     </row>
     <row r="8">
@@ -1232,22 +1232,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>161</v>
+        <v>147</v>
       </c>
       <c r="C8" t="n">
-        <v>35.28</v>
+        <v>35.85</v>
       </c>
       <c r="D8" t="n">
-        <v>22.8</v>
+        <v>22.07</v>
       </c>
       <c r="E8" t="n">
-        <v>6.529999999999999</v>
+        <v>6.59</v>
       </c>
       <c r="F8" t="n">
-        <v>21.773</v>
+        <v>21.9819</v>
       </c>
       <c r="G8" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H8" t="n">
         <v>51</v>
@@ -1259,13 +1259,13 @@
         <v>17</v>
       </c>
       <c r="K8" t="n">
-        <v>7.06</v>
+        <v>6.66</v>
       </c>
       <c r="L8" t="n">
-        <v>1.3558</v>
+        <v>1.3571</v>
       </c>
       <c r="M8" t="n">
-        <v>1.152</v>
+        <v>1.1672</v>
       </c>
     </row>
     <row r="9">
@@ -1275,25 +1275,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>140</v>
+        <v>175</v>
       </c>
       <c r="C9" t="n">
-        <v>31.99</v>
+        <v>37.61</v>
       </c>
       <c r="D9" t="n">
-        <v>20.58</v>
+        <v>23.53</v>
       </c>
       <c r="E9" t="n">
-        <v>5.899999999999999</v>
+        <v>7.03</v>
       </c>
       <c r="F9" t="n">
-        <v>19.6516</v>
+        <v>23.433</v>
       </c>
       <c r="G9" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="H9" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I9" t="n">
         <v>17</v>
@@ -1302,13 +1302,13 @@
         <v>17</v>
       </c>
       <c r="K9" t="n">
-        <v>6.8</v>
+        <v>7.44</v>
       </c>
       <c r="L9" t="n">
-        <v>1.3437</v>
+        <v>1.3637</v>
       </c>
       <c r="M9" t="n">
-        <v>1.2069</v>
+        <v>1.1641</v>
       </c>
     </row>
   </sheetData>
@@ -1399,22 +1399,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C2" t="n">
-        <v>30.09</v>
+        <v>35.24</v>
       </c>
       <c r="D2" t="n">
-        <v>14.3</v>
+        <v>16.17</v>
       </c>
       <c r="E2" t="n">
-        <v>5.46</v>
+        <v>6.569999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>18.2163</v>
+        <v>21.8925</v>
       </c>
       <c r="G2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H2" t="n">
         <v>53</v>
@@ -1426,13 +1426,13 @@
         <v>17</v>
       </c>
       <c r="K2" t="n">
-        <v>7.27</v>
+        <v>7.3</v>
       </c>
       <c r="L2" t="n">
-        <v>1.3885</v>
+        <v>1.4114</v>
       </c>
       <c r="M2" t="n">
-        <v>1.1565</v>
+        <v>1.1597</v>
       </c>
     </row>
     <row r="3">
@@ -1442,40 +1442,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C3" t="n">
-        <v>31.83</v>
+        <v>34.68</v>
       </c>
       <c r="D3" t="n">
-        <v>15.12</v>
+        <v>15.82</v>
       </c>
       <c r="E3" t="n">
-        <v>5.77</v>
+        <v>6.21</v>
       </c>
       <c r="F3" t="n">
-        <v>19.2357</v>
+        <v>20.7007</v>
       </c>
       <c r="G3" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H3" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J3" t="n">
         <v>17</v>
       </c>
       <c r="K3" t="n">
-        <v>6.42</v>
+        <v>6.51</v>
       </c>
       <c r="L3" t="n">
-        <v>1.3982</v>
+        <v>1.401</v>
       </c>
       <c r="M3" t="n">
-        <v>1.1535</v>
+        <v>1.1588</v>
       </c>
     </row>
     <row r="4">
@@ -1485,25 +1485,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="C4" t="n">
-        <v>34.14</v>
+        <v>30.18</v>
       </c>
       <c r="D4" t="n">
-        <v>16.23</v>
+        <v>13.93</v>
       </c>
       <c r="E4" t="n">
-        <v>6.22</v>
+        <v>5.47</v>
       </c>
       <c r="F4" t="n">
-        <v>20.7181</v>
+        <v>18.2417</v>
       </c>
       <c r="G4" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H4" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I4" t="n">
         <v>17</v>
@@ -1512,13 +1512,13 @@
         <v>17</v>
       </c>
       <c r="K4" t="n">
-        <v>6.47</v>
+        <v>6.68</v>
       </c>
       <c r="L4" t="n">
-        <v>1.3751</v>
+        <v>1.3837</v>
       </c>
       <c r="M4" t="n">
-        <v>1.1694</v>
+        <v>1.1801</v>
       </c>
     </row>
     <row r="5">
@@ -1528,40 +1528,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C5" t="n">
-        <v>29.49</v>
+        <v>34.46</v>
       </c>
       <c r="D5" t="n">
-        <v>13.5</v>
+        <v>16.41</v>
       </c>
       <c r="E5" t="n">
-        <v>5.3</v>
+        <v>6.29</v>
       </c>
       <c r="F5" t="n">
-        <v>17.6773</v>
+        <v>20.9526</v>
       </c>
       <c r="G5" t="n">
         <v>71</v>
       </c>
       <c r="H5" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="I5" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J5" t="n">
         <v>17</v>
       </c>
       <c r="K5" t="n">
-        <v>5.41</v>
+        <v>5.85</v>
       </c>
       <c r="L5" t="n">
-        <v>1.3814</v>
+        <v>1.3826</v>
       </c>
       <c r="M5" t="n">
-        <v>1.2075</v>
+        <v>1.1756</v>
       </c>
     </row>
     <row r="6">
@@ -1571,25 +1571,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C6" t="n">
-        <v>33.07</v>
+        <v>31.3</v>
       </c>
       <c r="D6" t="n">
-        <v>15.71</v>
+        <v>15.14</v>
       </c>
       <c r="E6" t="n">
-        <v>6.17</v>
+        <v>5.779999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>20.5525</v>
+        <v>19.2611</v>
       </c>
       <c r="G6" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H6" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I6" t="n">
         <v>16</v>
@@ -1598,13 +1598,13 @@
         <v>17</v>
       </c>
       <c r="K6" t="n">
-        <v>5.54</v>
+        <v>5.81</v>
       </c>
       <c r="L6" t="n">
-        <v>1.4009</v>
+        <v>1.3954</v>
       </c>
       <c r="M6" t="n">
-        <v>1.1842</v>
+        <v>1.1859</v>
       </c>
     </row>
     <row r="7">
@@ -1614,25 +1614,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="C7" t="n">
-        <v>33.61</v>
+        <v>30.65</v>
       </c>
       <c r="D7" t="n">
-        <v>15.12</v>
+        <v>14.82</v>
       </c>
       <c r="E7" t="n">
-        <v>6.140000000000001</v>
+        <v>5.67</v>
       </c>
       <c r="F7" t="n">
-        <v>20.4766</v>
+        <v>18.8878</v>
       </c>
       <c r="G7" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H7" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I7" t="n">
         <v>17</v>
@@ -1641,13 +1641,13 @@
         <v>17</v>
       </c>
       <c r="K7" t="n">
-        <v>6.35</v>
+        <v>7.09</v>
       </c>
       <c r="L7" t="n">
-        <v>1.3987</v>
+        <v>1.3972</v>
       </c>
       <c r="M7" t="n">
-        <v>1.1826</v>
+        <v>1.1742</v>
       </c>
     </row>
     <row r="8">
@@ -1657,40 +1657,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="C8" t="n">
-        <v>31.81</v>
+        <v>34.63</v>
       </c>
       <c r="D8" t="n">
-        <v>14.67</v>
+        <v>17.08</v>
       </c>
       <c r="E8" t="n">
-        <v>5.94</v>
+        <v>6.52</v>
       </c>
       <c r="F8" t="n">
-        <v>19.7964</v>
+        <v>21.7438</v>
       </c>
       <c r="G8" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H8" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I8" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J8" t="n">
         <v>17</v>
       </c>
       <c r="K8" t="n">
-        <v>6.61</v>
+        <v>6.26</v>
       </c>
       <c r="L8" t="n">
-        <v>1.3925</v>
+        <v>1.39</v>
       </c>
       <c r="M8" t="n">
-        <v>1.1989</v>
+        <v>1.1967</v>
       </c>
     </row>
     <row r="9">
@@ -1700,40 +1700,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="C9" t="n">
-        <v>35.48</v>
+        <v>32.98</v>
       </c>
       <c r="D9" t="n">
-        <v>16.94</v>
+        <v>14.66</v>
       </c>
       <c r="E9" t="n">
-        <v>6.47</v>
+        <v>5.93</v>
       </c>
       <c r="F9" t="n">
-        <v>21.5717</v>
+        <v>19.7825</v>
       </c>
       <c r="G9" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H9" t="n">
         <v>50</v>
       </c>
       <c r="I9" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J9" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K9" t="n">
-        <v>6.79</v>
+        <v>7.37</v>
       </c>
       <c r="L9" t="n">
-        <v>1.3838</v>
+        <v>1.3962</v>
       </c>
       <c r="M9" t="n">
-        <v>1.1793</v>
+        <v>1.1637</v>
       </c>
     </row>
     <row r="10">
@@ -1743,40 +1743,40 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>251</v>
+        <v>238</v>
       </c>
       <c r="C10" t="n">
-        <v>35.56</v>
+        <v>35.53</v>
       </c>
       <c r="D10" t="n">
-        <v>34.06</v>
+        <v>32.04</v>
       </c>
       <c r="E10" t="n">
-        <v>6.510000000000001</v>
+        <v>6.5</v>
       </c>
       <c r="F10" t="n">
-        <v>21.6902</v>
+        <v>21.6527</v>
       </c>
       <c r="G10" t="n">
         <v>62</v>
       </c>
       <c r="H10" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K10" t="n">
-        <v>7.37</v>
+        <v>7.43</v>
       </c>
       <c r="L10" t="n">
-        <v>1.4135</v>
+        <v>1.4126</v>
       </c>
       <c r="M10" t="n">
-        <v>1.1585</v>
+        <v>1.1574</v>
       </c>
     </row>
     <row r="11">
@@ -1786,25 +1786,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="C11" t="n">
-        <v>33.94</v>
+        <v>34.42</v>
       </c>
       <c r="D11" t="n">
-        <v>31.78</v>
+        <v>33.12</v>
       </c>
       <c r="E11" t="n">
-        <v>6.239999999999999</v>
+        <v>6.329999999999999</v>
       </c>
       <c r="F11" t="n">
-        <v>20.7966</v>
+        <v>21.104</v>
       </c>
       <c r="G11" t="n">
         <v>70</v>
       </c>
       <c r="H11" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I11" t="n">
         <v>17</v>
@@ -1813,13 +1813,13 @@
         <v>17</v>
       </c>
       <c r="K11" t="n">
-        <v>5.79</v>
+        <v>6.04</v>
       </c>
       <c r="L11" t="n">
-        <v>1.4136</v>
+        <v>1.4095</v>
       </c>
       <c r="M11" t="n">
-        <v>1.1844</v>
+        <v>1.1773</v>
       </c>
     </row>
   </sheetData>
@@ -1910,40 +1910,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="C2" t="n">
-        <v>24.04</v>
+        <v>22.01</v>
       </c>
       <c r="D2" t="n">
-        <v>11.42</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>4.36</v>
+        <v>3.81</v>
       </c>
       <c r="F2" t="n">
-        <v>14.5394</v>
+        <v>12.6855</v>
       </c>
       <c r="G2" t="n">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="H2" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="I2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J2" t="n">
         <v>18</v>
       </c>
       <c r="K2" t="n">
-        <v>6.04</v>
+        <v>4.52</v>
       </c>
       <c r="L2" t="n">
-        <v>1.2076</v>
+        <v>1.1806</v>
       </c>
       <c r="M2" t="n">
-        <v>1.1964</v>
+        <v>1.1459</v>
       </c>
     </row>
     <row r="3">
@@ -1953,22 +1953,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>371</v>
+        <v>403</v>
       </c>
       <c r="C3" t="n">
-        <v>36.62</v>
+        <v>37.49</v>
       </c>
       <c r="D3" t="n">
-        <v>52.95</v>
+        <v>54.37</v>
       </c>
       <c r="E3" t="n">
-        <v>6.74</v>
+        <v>6.92</v>
       </c>
       <c r="F3" t="n">
-        <v>22.4721</v>
+        <v>23.0753</v>
       </c>
       <c r="G3" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H3" t="n">
         <v>50</v>
@@ -1980,13 +1980,13 @@
         <v>17</v>
       </c>
       <c r="K3" t="n">
-        <v>7.01</v>
+        <v>7.41</v>
       </c>
       <c r="L3" t="n">
-        <v>1.423</v>
+        <v>1.4272</v>
       </c>
       <c r="M3" t="n">
-        <v>1.1583</v>
+        <v>1.1557</v>
       </c>
     </row>
     <row r="4">
@@ -1996,22 +1996,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="C4" t="n">
-        <v>33.46</v>
+        <v>33.56</v>
       </c>
       <c r="D4" t="n">
-        <v>77.48</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>6.13</v>
+        <v>6.18</v>
       </c>
       <c r="F4" t="n">
-        <v>20.4377</v>
+        <v>20.5842</v>
       </c>
       <c r="G4" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H4" t="n">
         <v>54</v>
@@ -2023,13 +2023,13 @@
         <v>17</v>
       </c>
       <c r="K4" t="n">
-        <v>6.14</v>
+        <v>6.16</v>
       </c>
       <c r="L4" t="n">
-        <v>1.4753</v>
+        <v>1.4768</v>
       </c>
       <c r="M4" t="n">
-        <v>1.1846</v>
+        <v>1.1855</v>
       </c>
     </row>
   </sheetData>
@@ -2120,40 +2120,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>101</v>
+        <v>70</v>
       </c>
       <c r="C2" t="n">
-        <v>31.71</v>
+        <v>34.17</v>
       </c>
       <c r="D2" t="n">
-        <v>15.75</v>
+        <v>11.59</v>
       </c>
       <c r="E2" t="n">
-        <v>5.79</v>
+        <v>6.19</v>
       </c>
       <c r="F2" t="n">
-        <v>19.3136</v>
+        <v>20.6168</v>
       </c>
       <c r="G2" t="n">
         <v>66</v>
       </c>
       <c r="H2" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="I2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J2" t="n">
         <v>17</v>
       </c>
       <c r="K2" t="n">
-        <v>6.41</v>
+        <v>6.04</v>
       </c>
       <c r="L2" t="n">
-        <v>1.4073</v>
+        <v>1.3799</v>
       </c>
       <c r="M2" t="n">
-        <v>1.1784</v>
+        <v>1.1781</v>
       </c>
     </row>
     <row r="3">
@@ -2163,25 +2163,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>96</v>
+        <v>62</v>
       </c>
       <c r="C3" t="n">
-        <v>32.89</v>
+        <v>33.93</v>
       </c>
       <c r="D3" t="n">
-        <v>16.91</v>
+        <v>12.13</v>
       </c>
       <c r="E3" t="n">
-        <v>5.81</v>
+        <v>5.800000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>19.3767</v>
+        <v>19.3419</v>
       </c>
       <c r="G3" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H3" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I3" t="n">
         <v>18</v>
@@ -2190,13 +2190,13 @@
         <v>18</v>
       </c>
       <c r="K3" t="n">
-        <v>5.68</v>
+        <v>5.11</v>
       </c>
       <c r="L3" t="n">
-        <v>1.4203</v>
+        <v>1.3865</v>
       </c>
       <c r="M3" t="n">
-        <v>1.1884</v>
+        <v>1.2085</v>
       </c>
     </row>
     <row r="4">
@@ -2206,40 +2206,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>107</v>
+        <v>67</v>
       </c>
       <c r="C4" t="n">
-        <v>34.04</v>
+        <v>31.89</v>
       </c>
       <c r="D4" t="n">
-        <v>17.93</v>
+        <v>11.95</v>
       </c>
       <c r="E4" t="n">
-        <v>6.18</v>
+        <v>5.7</v>
       </c>
       <c r="F4" t="n">
-        <v>20.59</v>
+        <v>19.0018</v>
       </c>
       <c r="G4" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="H4" t="n">
         <v>49</v>
       </c>
       <c r="I4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J4" t="n">
         <v>17</v>
       </c>
       <c r="K4" t="n">
-        <v>5.97</v>
+        <v>5.61</v>
       </c>
       <c r="L4" t="n">
-        <v>1.4048</v>
+        <v>1.3878</v>
       </c>
       <c r="M4" t="n">
-        <v>1.1719</v>
+        <v>1.1961</v>
       </c>
     </row>
     <row r="5">
@@ -2249,40 +2249,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60</v>
+        <v>104</v>
       </c>
       <c r="C5" t="n">
-        <v>32.02999999999999</v>
+        <v>34.19</v>
       </c>
       <c r="D5" t="n">
-        <v>11.6</v>
+        <v>17.4</v>
       </c>
       <c r="E5" t="n">
-        <v>5.54</v>
+        <v>5.99</v>
       </c>
       <c r="F5" t="n">
-        <v>18.4547</v>
+        <v>19.9829</v>
       </c>
       <c r="G5" t="n">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H5" t="n">
         <v>55</v>
       </c>
       <c r="I5" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J5" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K5" t="n">
-        <v>5.17</v>
+        <v>5.98</v>
       </c>
       <c r="L5" t="n">
-        <v>1.3833</v>
+        <v>1.4</v>
       </c>
       <c r="M5" t="n">
-        <v>1.2838</v>
+        <v>1.2161</v>
       </c>
     </row>
     <row r="6">
@@ -2292,25 +2292,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>63</v>
+        <v>94</v>
       </c>
       <c r="C6" t="n">
-        <v>32.88</v>
+        <v>31.29</v>
       </c>
       <c r="D6" t="n">
-        <v>12.58</v>
+        <v>17</v>
       </c>
       <c r="E6" t="n">
-        <v>6.02</v>
+        <v>5.84</v>
       </c>
       <c r="F6" t="n">
-        <v>20.0559</v>
+        <v>19.4826</v>
       </c>
       <c r="G6" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H6" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="I6" t="n">
         <v>17</v>
@@ -2319,13 +2319,13 @@
         <v>17</v>
       </c>
       <c r="K6" t="n">
-        <v>5.01</v>
+        <v>5.53</v>
       </c>
       <c r="L6" t="n">
-        <v>1.3892</v>
+        <v>1.4191</v>
       </c>
       <c r="M6" t="n">
-        <v>1.2131</v>
+        <v>1.1862</v>
       </c>
     </row>
     <row r="7">
@@ -2335,25 +2335,25 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>98</v>
+      </c>
+      <c r="C7" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="D7" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="F7" t="n">
+        <v>19.2103</v>
+      </c>
+      <c r="G7" t="n">
         <v>67</v>
       </c>
-      <c r="C7" t="n">
-        <v>32.71</v>
-      </c>
-      <c r="D7" t="n">
-        <v>11.44</v>
-      </c>
-      <c r="E7" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="F7" t="n">
-        <v>20.3425</v>
-      </c>
-      <c r="G7" t="n">
-        <v>66</v>
-      </c>
       <c r="H7" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="I7" t="n">
         <v>18</v>
@@ -2362,13 +2362,13 @@
         <v>17</v>
       </c>
       <c r="K7" t="n">
-        <v>5.86</v>
+        <v>6.26</v>
       </c>
       <c r="L7" t="n">
-        <v>1.3755</v>
+        <v>1.4067</v>
       </c>
       <c r="M7" t="n">
-        <v>1.202</v>
+        <v>1.1848</v>
       </c>
     </row>
     <row r="8">
@@ -2378,40 +2378,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="C8" t="n">
-        <v>32.76</v>
+        <v>33.11</v>
       </c>
       <c r="D8" t="n">
-        <v>11.5</v>
+        <v>16.96</v>
       </c>
       <c r="E8" t="n">
-        <v>6.12</v>
+        <v>6.25</v>
       </c>
       <c r="F8" t="n">
-        <v>20.4076</v>
+        <v>20.8301</v>
       </c>
       <c r="G8" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="H8" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I8" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J8" t="n">
         <v>17</v>
       </c>
       <c r="K8" t="n">
-        <v>6.17</v>
+        <v>5.6</v>
       </c>
       <c r="L8" t="n">
-        <v>1.378</v>
+        <v>1.3903</v>
       </c>
       <c r="M8" t="n">
-        <v>1.1872</v>
+        <v>1.2001</v>
       </c>
     </row>
     <row r="9">
@@ -2421,19 +2421,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="C9" t="n">
-        <v>33.06</v>
+        <v>33.39</v>
       </c>
       <c r="D9" t="n">
-        <v>16.15</v>
+        <v>11.12</v>
       </c>
       <c r="E9" t="n">
-        <v>5.949999999999999</v>
+        <v>5.92</v>
       </c>
       <c r="F9" t="n">
-        <v>19.8347</v>
+        <v>19.7295</v>
       </c>
       <c r="G9" t="n">
         <v>67</v>
@@ -2442,19 +2442,19 @@
         <v>52</v>
       </c>
       <c r="I9" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J9" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K9" t="n">
-        <v>6.01</v>
+        <v>6.21</v>
       </c>
       <c r="L9" t="n">
-        <v>1.3831</v>
+        <v>1.3728</v>
       </c>
       <c r="M9" t="n">
-        <v>1.1808</v>
+        <v>1.1809</v>
       </c>
     </row>
     <row r="10">
@@ -2464,25 +2464,25 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>377</v>
+        <v>312</v>
       </c>
       <c r="C10" t="n">
-        <v>33.2</v>
+        <v>34.22</v>
       </c>
       <c r="D10" t="n">
-        <v>62.91</v>
+        <v>54.38</v>
       </c>
       <c r="E10" t="n">
-        <v>5.92</v>
+        <v>6.069999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>19.7359</v>
+        <v>20.2223</v>
       </c>
       <c r="G10" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H10" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I10" t="n">
         <v>18</v>
@@ -2491,13 +2491,13 @@
         <v>17</v>
       </c>
       <c r="K10" t="n">
-        <v>5.99</v>
+        <v>5.74</v>
       </c>
       <c r="L10" t="n">
-        <v>1.5142</v>
+        <v>1.4939</v>
       </c>
       <c r="M10" t="n">
-        <v>1.1928</v>
+        <v>1.2018</v>
       </c>
     </row>
     <row r="11">
@@ -2507,25 +2507,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>307</v>
+        <v>379</v>
       </c>
       <c r="C11" t="n">
-        <v>33.27</v>
+        <v>32.82</v>
       </c>
       <c r="D11" t="n">
-        <v>52.51</v>
+        <v>62.23</v>
       </c>
       <c r="E11" t="n">
-        <v>6.140000000000001</v>
+        <v>6.09</v>
       </c>
       <c r="F11" t="n">
-        <v>20.4516</v>
+        <v>20.2962</v>
       </c>
       <c r="G11" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H11" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="I11" t="n">
         <v>18</v>
@@ -2534,13 +2534,13 @@
         <v>17</v>
       </c>
       <c r="K11" t="n">
-        <v>5.85</v>
+        <v>6.09</v>
       </c>
       <c r="L11" t="n">
-        <v>1.4862</v>
+        <v>1.5118</v>
       </c>
       <c r="M11" t="n">
-        <v>1.1932</v>
+        <v>1.1841</v>
       </c>
     </row>
     <row r="12">
@@ -2550,22 +2550,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>207</v>
+        <v>136</v>
       </c>
       <c r="C12" t="n">
-        <v>34.32</v>
+        <v>34.25</v>
       </c>
       <c r="D12" t="n">
-        <v>35.72</v>
+        <v>25.32</v>
       </c>
       <c r="E12" t="n">
-        <v>6.15</v>
+        <v>6.05</v>
       </c>
       <c r="F12" t="n">
-        <v>20.4884</v>
+        <v>20.1549</v>
       </c>
       <c r="G12" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H12" t="n">
         <v>54</v>
@@ -2577,13 +2577,13 @@
         <v>17</v>
       </c>
       <c r="K12" t="n">
-        <v>5.8</v>
+        <v>5.37</v>
       </c>
       <c r="L12" t="n">
-        <v>1.4241</v>
+        <v>1.3894</v>
       </c>
       <c r="M12" t="n">
-        <v>1.178</v>
+        <v>1.2012</v>
       </c>
     </row>
     <row r="13">
@@ -2593,40 +2593,40 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>144</v>
+        <v>212</v>
       </c>
       <c r="C13" t="n">
-        <v>33.65000000000001</v>
+        <v>33.44</v>
       </c>
       <c r="D13" t="n">
-        <v>23.59</v>
+        <v>34.32</v>
       </c>
       <c r="E13" t="n">
-        <v>6.279999999999999</v>
+        <v>6.32</v>
       </c>
       <c r="F13" t="n">
-        <v>20.949</v>
+        <v>21.0574</v>
       </c>
       <c r="G13" t="n">
         <v>69</v>
       </c>
       <c r="H13" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I13" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J13" t="n">
         <v>17</v>
       </c>
       <c r="K13" t="n">
-        <v>6.1</v>
+        <v>6.18</v>
       </c>
       <c r="L13" t="n">
-        <v>1.3747</v>
+        <v>1.4154</v>
       </c>
       <c r="M13" t="n">
-        <v>1.1921</v>
+        <v>1.1892</v>
       </c>
     </row>
     <row r="14">
@@ -2636,25 +2636,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>137</v>
+        <v>207</v>
       </c>
       <c r="C14" t="n">
-        <v>34.03</v>
+        <v>33.73</v>
       </c>
       <c r="D14" t="n">
-        <v>25.46</v>
+        <v>35.6</v>
       </c>
       <c r="E14" t="n">
-        <v>6.08</v>
+        <v>6.13</v>
       </c>
       <c r="F14" t="n">
-        <v>20.2665</v>
+        <v>20.4172</v>
       </c>
       <c r="G14" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="H14" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I14" t="n">
         <v>18</v>
@@ -2663,13 +2663,13 @@
         <v>17</v>
       </c>
       <c r="K14" t="n">
-        <v>5.38</v>
+        <v>5.81</v>
       </c>
       <c r="L14" t="n">
-        <v>1.3915</v>
+        <v>1.4255</v>
       </c>
       <c r="M14" t="n">
-        <v>1.2394</v>
+        <v>1.1959</v>
       </c>
     </row>
     <row r="15">
@@ -2679,37 +2679,37 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>211</v>
+        <v>144</v>
       </c>
       <c r="C15" t="n">
-        <v>33.93</v>
+        <v>34.53</v>
       </c>
       <c r="D15" t="n">
-        <v>33.38</v>
+        <v>23.41</v>
       </c>
       <c r="E15" t="n">
-        <v>6.140000000000001</v>
+        <v>6.239999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>20.4816</v>
+        <v>20.7941</v>
       </c>
       <c r="G15" t="n">
         <v>66</v>
       </c>
       <c r="H15" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I15" t="n">
         <v>18</v>
       </c>
       <c r="J15" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K15" t="n">
-        <v>6.32</v>
+        <v>6.15</v>
       </c>
       <c r="L15" t="n">
-        <v>1.412</v>
+        <v>1.376</v>
       </c>
       <c r="M15" t="n">
         <v>1.176</v>
@@ -2722,25 +2722,25 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>710</v>
+        <v>704</v>
       </c>
       <c r="C16" t="n">
-        <v>34.01</v>
+        <v>33.92</v>
       </c>
       <c r="D16" t="n">
-        <v>118.31</v>
+        <v>118.16</v>
       </c>
       <c r="E16" t="n">
-        <v>6.17</v>
+        <v>6.16</v>
       </c>
       <c r="F16" t="n">
-        <v>20.5568</v>
+        <v>20.5307</v>
       </c>
       <c r="G16" t="n">
         <v>70</v>
       </c>
       <c r="H16" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I16" t="n">
         <v>18</v>
@@ -2749,13 +2749,13 @@
         <v>17</v>
       </c>
       <c r="K16" t="n">
-        <v>6</v>
+        <v>5.96</v>
       </c>
       <c r="L16" t="n">
-        <v>1.5506</v>
+        <v>1.5513</v>
       </c>
       <c r="M16" t="n">
-        <v>1.1928</v>
+        <v>1.1945</v>
       </c>
     </row>
   </sheetData>

</xml_diff>